<commit_message>
Step 2: assumption tests and Kruskal-Conover analysis
</commit_message>
<xml_diff>
--- a/analysis_outputs/step_02/Table_06_Kruskal_Omnibus.xlsx
+++ b/analysis_outputs/step_02/Table_06_Kruskal_Omnibus.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,11 @@
           <t>p_value</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Omnibus_significant_p_lt_0_05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,6 +494,9 @@
       <c r="G2" t="n">
         <v>5.50811847483888e-07</v>
       </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,6 +522,9 @@
       <c r="G3" t="n">
         <v>5.192968590027221e-11</v>
       </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -539,6 +550,9 @@
       <c r="G4" t="n">
         <v>1.43001591743226e-10</v>
       </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -564,6 +578,9 @@
       <c r="G5" t="n">
         <v>4.294382094017315e-07</v>
       </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -589,6 +606,9 @@
       <c r="G6" t="n">
         <v>5.150350749945782e-09</v>
       </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -614,6 +634,9 @@
       <c r="G7" t="n">
         <v>8.502627440347e-09</v>
       </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -639,6 +662,9 @@
       <c r="G8" t="n">
         <v>0.003201216236313163</v>
       </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -664,6 +690,9 @@
       <c r="G9" t="n">
         <v>0.05569451743392675</v>
       </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -688,6 +717,9 @@
       </c>
       <c r="G10" t="n">
         <v>0.5089791919988667</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>